<commit_message>
chore(sync): 2026-10-30 push local changes from PC2 (sync to PC3)
</commit_message>
<xml_diff>
--- a/assets/registry/ledgers/ShellStorm2_敌人账本_v001.xlsx
+++ b/assets/registry/ledgers/ShellStorm2_敌人账本_v001.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="总览" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="账本说明" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="资产主表" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="敌人动画与状态" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="3D-敌人" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="域变更日志" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="总览" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="账本说明" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="资产主表" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="敌人动画与状态" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3D-敌人" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="域变更日志" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'资产主表'!$A$5:$Y$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'资产主表'!$A$5:$Y$54</definedName>
   </definedNames>
-  <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.001"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -1307,22 +1307,22 @@
     </row>
     <row r="6" ht="42" customHeight="1" s="38">
       <c r="A6" s="43">
-        <f>COUNTA('资产主表'!$A$6:$A$53)</f>
+        <f>COUNTA('资产主表'!$A$6:$A$54)</f>
         <v/>
       </c>
       <c r="B6" s="41" t="n"/>
       <c r="C6" s="43">
-        <f>COUNTIF('资产主表'!$K$6:$K$53,"已完成")+COUNTIF('资产主表'!$K$6:$K$53,"原型已接入")+COUNTIF('资产主表'!$K$6:$K$53,"正式美术已接入")+COUNTIF('资产主表'!$K$6:$K$53,"已优化并正式接入")+COUNTIF('资产主表'!$K$6:$K$53,"Blender源已完成")+COUNTIF('资产主表'!$K$6:$K$53,"已导入；优化完成")+COUNTIF('资产主表'!$K$6:$K$53,"白模源已完成；QA PASS")</f>
+        <f>COUNTIF('资产主表'!$K$6:$K$54,"已完成")+COUNTIF('资产主表'!$K$6:$K$54,"原型已接入")+COUNTIF('资产主表'!$K$6:$K$54,"正式美术已接入")+COUNTIF('资产主表'!$K$6:$K$54,"已优化并正式接入")+COUNTIF('资产主表'!$K$6:$K$54,"Blender源已完成")+COUNTIF('资产主表'!$K$6:$K$54,"已导入；优化完成")+COUNTIF('资产主表'!$K$6:$K$54,"白模源已完成；QA PASS")</f>
         <v/>
       </c>
       <c r="D6" s="41" t="n"/>
       <c r="E6" s="43">
-        <f>COUNTIF('资产主表'!$K$6:$K$53,"待制作")+COUNTIF('资产主表'!$K$6:$K$53,"程序占位")</f>
+        <f>COUNTIF('资产主表'!$K$6:$K$54,"待制作")+COUNTIF('资产主表'!$K$6:$K$54,"程序占位")</f>
         <v/>
       </c>
       <c r="F6" s="41" t="n"/>
       <c r="G6" s="43">
-        <f>COUNTIF('资产主表'!$S$6:$S$53,"重复")</f>
+        <f>COUNTIF('资产主表'!$S$6:$S$54,"重复")</f>
         <v/>
       </c>
       <c r="H6" s="41" t="n"/>
@@ -1391,11 +1391,11 @@
         </is>
       </c>
       <c r="B10" s="48">
-        <f>COUNTIF('资产主表'!$C$6:$C$53,A10)</f>
+        <f>COUNTIF('资产主表'!$C$6:$C$54,A10)</f>
         <v/>
       </c>
       <c r="C10" s="48">
-        <f>SUMPRODUCT(('资产主表'!$C$6:$C$53=A10)*(('资产主表'!$K$6:$K$53="已完成")+('资产主表'!$K$6:$K$53="原型已接入")+('资产主表'!$K$6:$K$53="正式美术已接入")+('资产主表'!$K$6:$K$53="已优化并正式接入")+('资产主表'!$K$6:$K$53="Blender源已完成")+('资产主表'!$K$6:$K$53="已导入；优化完成")+('资产主表'!$K$6:$K$53="白模源已完成；QA PASS")))</f>
+        <f>SUMPRODUCT(('资产主表'!$C$6:$C$54=A10)*(('资产主表'!$K$6:$K$54="已完成")+('资产主表'!$K$6:$K$54="原型已接入")+('资产主表'!$K$6:$K$54="正式美术已接入")+('资产主表'!$K$6:$K$54="已优化并正式接入")+('资产主表'!$K$6:$K$54="Blender源已完成")+('资产主表'!$K$6:$K$54="已导入；优化完成")+('资产主表'!$K$6:$K$54="白模源已完成；QA PASS")))</f>
         <v/>
       </c>
       <c r="D10" s="48" t="n"/>
@@ -1413,11 +1413,11 @@
         </is>
       </c>
       <c r="B11" s="44">
-        <f>COUNTIF('资产主表'!$C$6:$C$53,A11)</f>
+        <f>COUNTIF('资产主表'!$C$6:$C$54,A11)</f>
         <v/>
       </c>
       <c r="C11" s="44">
-        <f>SUMPRODUCT(('资产主表'!$C$6:$C$53=A11)*(('资产主表'!$K$6:$K$53="已完成")+('资产主表'!$K$6:$K$53="原型已接入")+('资产主表'!$K$6:$K$53="正式美术已接入")+('资产主表'!$K$6:$K$53="已优化并正式接入")+('资产主表'!$K$6:$K$53="Blender源已完成")+('资产主表'!$K$6:$K$53="已导入；优化完成")+('资产主表'!$K$6:$K$53="白模源已完成；QA PASS")))</f>
+        <f>SUMPRODUCT(('资产主表'!$C$6:$C$54=A11)*(('资产主表'!$K$6:$K$54="已完成")+('资产主表'!$K$6:$K$54="原型已接入")+('资产主表'!$K$6:$K$54="正式美术已接入")+('资产主表'!$K$6:$K$54="已优化并正式接入")+('资产主表'!$K$6:$K$54="Blender源已完成")+('资产主表'!$K$6:$K$54="已导入；优化完成")+('资产主表'!$K$6:$K$54="白模源已完成；QA PASS")))</f>
         <v/>
       </c>
       <c r="D11" s="44" t="n"/>
@@ -1965,7 +1965,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:Y53"/>
+  <dimension ref="A1:Y54"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="10.359375" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="29.84" customWidth="1" style="37" min="1" max="1"/>
@@ -2225,12 +2225,12 @@
       </c>
       <c r="M6" s="62" t="inlineStr">
         <is>
-          <t>v004</t>
+          <t>v005</t>
         </is>
       </c>
       <c r="N6" s="62" t="inlineStr">
         <is>
-          <t>游戏高1.3m；源高1.857143m；1790三角/897顶点；20骨；512贴图；6剪辑</t>
+          <t>名义展示1.3m/倍率0.70；静止绑定高1.893537m；800三角/402顶点；16骨；512贴图；6剪辑</t>
         </is>
       </c>
       <c r="O6" s="62" t="inlineStr">
@@ -2240,7 +2240,7 @@
       </c>
       <c r="P6" s="62" t="inlineStr">
         <is>
-          <t>art_source/enemies/normal_enemy_3d/melee_chaser/source/model/enm_melee_fungboar01_model_v003.blend; art_source/enemies/normal_enemy_3d/melee_chaser/source/animation/enm_melee_fungboar01_animation_v004.blend</t>
+          <t>art_source/enemies/normal_enemy_3d/melee_chaser/source/model/enm_melee_fungboar01_model_v004.blend; art_source/enemies/normal_enemy_3d/melee_chaser/source/animation/enm_melee_fungboar01_animation_v005.blend</t>
         </is>
       </c>
       <c r="Q6" s="49" t="inlineStr">
@@ -2253,12 +2253,12 @@
         <v/>
       </c>
       <c r="S6" s="49">
-        <f>IF(COUNTIF($R$6:$R$53,R6)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$54,R6)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T6" s="62" t="inlineStr">
         <is>
-          <t>6b88f60e398a204cc3d31719550138c7dad8866d0477fa41094ecb0c228b07c0</t>
+          <t>454c59f3f495f6b90402ba2041f9ed80262d51ed4f16db59d825804e612e552c</t>
         </is>
       </c>
       <c r="U6" s="62" t="inlineStr">
@@ -2266,8 +2266,10 @@
           <t>Codex</t>
         </is>
       </c>
-      <c r="V6" s="63" t="n">
-        <v>46304</v>
+      <c r="V6" s="63" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
       </c>
       <c r="W6" s="62" t="inlineStr">
         <is>
@@ -2285,7 +2287,8 @@
 2026-09-20 首个标准普通怪转正：Tripo 源 → Blender 重制（模型 v002 / 动作 v003），六段剪辑按 12 态采样，verify_melee_zombie_presentation 通过。
 显示名迁移：小菌猪 → 小僵尸（Enemy3D.configure_from_enemy_data 精确迁移旧存档尾名）；AssetID 与逻辑 ID 不变。
 未闭合：碰撞 FOOTPRINT_PROFILES(radius 1.02/height 1.30) 仍为旧程序网格口径，按新几何应为 0.641/1.857，属玩法数值待拍板；贴图仅 basecolor，无法线贴图。
-2026-10-09 v004减面与减骨：4552→1790三角，897顶点；36→20骨，移除16根手指骨，每手仅一根手骨；自然弯曲形状固定，手指权重合并至手骨并重新归一。512贴图/六段身体动作/12态/碰撞/受击闪色/2.4秒死亡保留。源重开、半帧蒙皮检查、运行专项及死亡视野真实渲染通过。</t>
+2026-10-09 v004减面与减骨：4552→1790三角，897顶点；36→20骨，移除16根手指骨，每手仅一根手骨；自然弯曲形状固定，手指权重合并至手骨并重新归一。512贴图/六段身体动作/12态/碰撞/受击闪色/2.4秒死亡保留。源重开、半帧蒙皮检查、运行专项及死亡视野真实渲染通过。
+2026-10-30 v005减面减骨：1790→800三角、402原生顶点，20→16骨；删除左右Hand/Foot骨，手指骨原已移除；手部随前臂、脚部随小腿，腕踝固定，不再独立弯曲。模型v004/动作v005，骨架SKEL-MELEE-ZOMBIE01-004（签名4b0767495dde049f663598129f285158dd04bdbe309ef2a66e042b8d6db033bb）；六剪辑时长/循环与12态采样保留。名义展示1.3m/倍率0.70不变；静止绑定脚底Z=0，高1.893537m；待机首姿源高1.800935m（展示约1.26065m），不能把静止绑定高度与姿势高度混为一谈。双源重开、1266个四分之一帧蒙皮/地面检查通过（最低Z≥0.0004999m、单位姿势、Root静止、循环接缝0），GLB六段时长精确。近景细节因减面简化；未进行全程自穿插、滑步及目标设备性能验收。运行专项exit0（12态/6剪辑/16骨/800三角/碰撞不变）；801面负向对照exit1且仅预期预算错误；120Hz运行时1266采样地面最低+0.00003319m、Root静止；存活12姿态及死亡可见性真实渲染均exit0，无非预期脚本错误。证据：ShellStorm2-work/sessions/2026-10-30_melee_800/；GLB SHA-256=800f1be604c65de3c0b669d0082b4e434f70dcebf70aa0b46918d643844ef775（172668字节），共享原有贴图。</t>
         </is>
       </c>
     </row>
@@ -2380,7 +2383,7 @@
         <v/>
       </c>
       <c r="S7" s="49">
-        <f>IF(COUNTIF($R$6:$R$53,R7)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$54,R7)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T7" s="62" t="inlineStr">
@@ -2495,7 +2498,7 @@
         <v/>
       </c>
       <c r="S8" s="49">
-        <f>IF(COUNTIF($R$6:$R$53,R8)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$54,R8)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T8" s="49" t="n"/>
@@ -2602,7 +2605,7 @@
         <v/>
       </c>
       <c r="S9" s="49">
-        <f>IF(COUNTIF($R$6:$R$53,R9)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$54,R9)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T9" s="49" t="n"/>
@@ -2713,7 +2716,7 @@
         <v/>
       </c>
       <c r="S10" s="49">
-        <f>IF(COUNTIF($R$6:$R$53,R10)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$54,R10)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T10" s="49" t="n"/>
@@ -2820,7 +2823,7 @@
         <v/>
       </c>
       <c r="S11" s="49">
-        <f>IF(COUNTIF($R$6:$R$53,R11)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$54,R11)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T11" s="49" t="n"/>
@@ -2927,7 +2930,7 @@
         <v/>
       </c>
       <c r="S12" s="49">
-        <f>IF(COUNTIF($R$6:$R$53,R12)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$54,R12)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T12" s="49" t="n"/>
@@ -3042,7 +3045,7 @@
         <v/>
       </c>
       <c r="S13" s="41">
-        <f>IF(COUNTIF($R$6:$R$53,R13)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$54,R13)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T13" s="65" t="inlineStr">
@@ -3161,7 +3164,7 @@
         <v/>
       </c>
       <c r="S14" s="41">
-        <f>IF(COUNTIF($R$6:$R$53,R14)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$54,R14)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T14" s="65" t="inlineStr">
@@ -3281,7 +3284,7 @@
         <v/>
       </c>
       <c r="S15" s="41">
-        <f>IF(COUNTIF($R$6:$R$53,R15)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$54,R15)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T15" s="65" t="inlineStr">
@@ -3401,7 +3404,7 @@
         <v/>
       </c>
       <c r="S16" s="41">
-        <f>IF(COUNTIF($R$6:$R$53,R16)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$54,R16)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T16" s="65" t="inlineStr">
@@ -3525,7 +3528,7 @@
         <v/>
       </c>
       <c r="S17" s="41">
-        <f>IF(COUNTIF($R$6:$R$53,R17)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$54,R17)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T17" s="65" t="inlineStr">
@@ -3642,7 +3645,7 @@
         <v/>
       </c>
       <c r="S18" s="49">
-        <f>IF(COUNTIF($R$6:$R$53,R18)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$54,R18)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T18" s="49" t="n"/>
@@ -3757,7 +3760,7 @@
         <v/>
       </c>
       <c r="S19" s="49">
-        <f>IF(COUNTIF($R$6:$R$53,R19)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$54,R19)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T19" s="49" t="inlineStr">
@@ -3876,7 +3879,7 @@
         <v/>
       </c>
       <c r="S20" s="49">
-        <f>IF(COUNTIF($R$6:$R$53,R20)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$54,R20)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T20" s="49" t="inlineStr">
@@ -4001,7 +4004,7 @@
         <v/>
       </c>
       <c r="S21" s="49">
-        <f>IF(COUNTIF($R$6:$R$53,R21)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$54,R21)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T21" s="49" t="inlineStr">
@@ -4126,7 +4129,7 @@
         <v/>
       </c>
       <c r="S22" s="49">
-        <f>IF(COUNTIF($R$6:$R$53,R22)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$54,R22)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T22" s="49" t="inlineStr">
@@ -4251,7 +4254,7 @@
         <v/>
       </c>
       <c r="S23" s="49">
-        <f>IF(COUNTIF($R$6:$R$53,R23)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$54,R23)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T23" s="49" t="inlineStr">
@@ -4376,7 +4379,7 @@
         <v/>
       </c>
       <c r="S24" s="49">
-        <f>IF(COUNTIF($R$6:$R$53,R24)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$54,R24)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T24" s="49" t="inlineStr">
@@ -4501,7 +4504,7 @@
         <v/>
       </c>
       <c r="S25" s="49">
-        <f>IF(COUNTIF($R$6:$R$53,R25)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$54,R25)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T25" s="49" t="inlineStr">
@@ -4626,7 +4629,7 @@
         <v/>
       </c>
       <c r="S26" s="49">
-        <f>IF(COUNTIF($R$6:$R$53,R26)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$54,R26)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T26" s="49" t="inlineStr">
@@ -4751,7 +4754,7 @@
         <v/>
       </c>
       <c r="S27" s="49">
-        <f>IF(COUNTIF($R$6:$R$53,R27)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$54,R27)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T27" s="49" t="inlineStr">
@@ -4876,7 +4879,7 @@
         <v/>
       </c>
       <c r="S28" s="49">
-        <f>IF(COUNTIF($R$6:$R$53,R28)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$54,R28)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T28" s="49" t="inlineStr">
@@ -4997,7 +5000,7 @@
         <v/>
       </c>
       <c r="S29" s="49">
-        <f>IF(COUNTIF($R$6:$R$53,R29)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$54,R29)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T29" s="49" t="inlineStr">
@@ -5118,7 +5121,7 @@
         <v/>
       </c>
       <c r="S30" s="49">
-        <f>IF(COUNTIF($R$6:$R$53,R30)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$54,R30)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T30" s="49" t="inlineStr">
@@ -5239,7 +5242,7 @@
         <v/>
       </c>
       <c r="S31" s="49">
-        <f>IF(COUNTIF($R$6:$R$53,R31)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$54,R31)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T31" s="49" t="inlineStr">
@@ -5360,7 +5363,7 @@
         <v/>
       </c>
       <c r="S32" s="49">
-        <f>IF(COUNTIF($R$6:$R$53,R32)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$54,R32)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T32" s="49" t="inlineStr">
@@ -5485,7 +5488,7 @@
         <v/>
       </c>
       <c r="S33" s="91">
-        <f>IF(COUNTIF($R$6:$R$53,R33)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$54,R33)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T33" s="91" t="inlineStr">
@@ -5610,7 +5613,7 @@
         <v/>
       </c>
       <c r="S34" s="91">
-        <f>IF(COUNTIF($R$6:$R$53,R34)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$54,R34)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T34" s="91" t="inlineStr">
@@ -5735,7 +5738,7 @@
         <v/>
       </c>
       <c r="S35" s="91">
-        <f>IF(COUNTIF($R$6:$R$53,R35)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$54,R35)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T35" s="91" t="inlineStr">
@@ -5856,7 +5859,7 @@
         <v/>
       </c>
       <c r="S36" s="91">
-        <f>IF(COUNTIF($R$6:$R$53,R36)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$54,R36)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T36" s="91" t="inlineStr">
@@ -5981,7 +5984,7 @@
         <v/>
       </c>
       <c r="S37" s="91">
-        <f>IF(COUNTIF($R$6:$R$53,R37)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$54,R37)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T37" s="91" t="inlineStr">
@@ -6102,7 +6105,7 @@
         <v/>
       </c>
       <c r="S38" s="91">
-        <f>IF(COUNTIF($R$6:$R$53,R38)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$54,R38)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T38" s="91" t="inlineStr">
@@ -6223,7 +6226,7 @@
         <v/>
       </c>
       <c r="S39" s="91">
-        <f>IF(COUNTIF($R$6:$R$53,R39)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$54,R39)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T39" s="91" t="inlineStr">
@@ -6344,7 +6347,7 @@
         <v/>
       </c>
       <c r="S40" s="91">
-        <f>IF(COUNTIF($R$6:$R$53,R40)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$54,R40)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T40" s="91" t="inlineStr">
@@ -6465,7 +6468,7 @@
         <v/>
       </c>
       <c r="S41" s="91">
-        <f>IF(COUNTIF($R$6:$R$53,R41)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$54,R41)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T41" s="91" t="inlineStr">
@@ -6586,7 +6589,7 @@
         <v/>
       </c>
       <c r="S42" s="91">
-        <f>IF(COUNTIF($R$6:$R$53,R42)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$54,R42)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T42" s="91" t="inlineStr">
@@ -6707,7 +6710,7 @@
         <v/>
       </c>
       <c r="S43" s="91">
-        <f>IF(COUNTIF($R$6:$R$53,R43)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$54,R43)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T43" s="91" t="inlineStr">
@@ -6828,7 +6831,7 @@
         <v/>
       </c>
       <c r="S44" s="91">
-        <f>IF(COUNTIF($R$6:$R$53,R44)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$54,R44)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T44" s="91" t="inlineStr">
@@ -6949,7 +6952,7 @@
         <v/>
       </c>
       <c r="S45" s="91">
-        <f>IF(COUNTIF($R$6:$R$53,R45)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$54,R45)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T45" s="91" t="inlineStr">
@@ -7074,7 +7077,7 @@
         <v/>
       </c>
       <c r="S46" s="91">
-        <f>IF(COUNTIF($R$6:$R$53,R46)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$54,R46)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T46" s="91" t="inlineStr">
@@ -7199,7 +7202,7 @@
         <v/>
       </c>
       <c r="S47" s="91">
-        <f>IF(COUNTIF($R$6:$R$53,R47)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$54,R47)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T47" s="91" t="inlineStr">
@@ -7324,7 +7327,7 @@
         <v/>
       </c>
       <c r="S48" s="91">
-        <f>IF(COUNTIF($R$6:$R$53,R48)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$54,R48)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T48" s="91" t="inlineStr">
@@ -7449,7 +7452,7 @@
         <v/>
       </c>
       <c r="S49" s="91">
-        <f>IF(COUNTIF($R$6:$R$53,R49)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$54,R49)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T49" s="91" t="inlineStr">
@@ -7574,7 +7577,7 @@
         <v/>
       </c>
       <c r="S50" s="91">
-        <f>IF(COUNTIF($R$6:$R$53,R50)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$54,R50)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T50" s="91" t="inlineStr">
@@ -7695,7 +7698,7 @@
         <v/>
       </c>
       <c r="S51" s="91">
-        <f>IF(COUNTIF($R$6:$R$53,R51)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$54,R51)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T51" s="91" t="inlineStr">
@@ -7820,7 +7823,7 @@
         <v/>
       </c>
       <c r="S52" s="91">
-        <f>IF(COUNTIF($R$6:$R$53,R52)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$54,R52)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T52" s="91" t="inlineStr">
@@ -7945,7 +7948,7 @@
         <v/>
       </c>
       <c r="S53" s="91">
-        <f>IF(COUNTIF($R$6:$R$53,R53)&gt;1,"重复","唯一")</f>
+        <f>IF(COUNTIF($R$6:$R$54,R53)&gt;1,"重复","唯一")</f>
         <v/>
       </c>
       <c r="T53" s="91" t="inlineStr">
@@ -7976,6 +7979,131 @@
       <c r="Y53" s="92" t="inlineStr">
         <is>
           <t>远征03《挺进地牢》第一层复刻怪（2026-10-29 第二批）。**本行是表现层占位**：复用 ENM-NORMAL-FAT-ZOMBIE03 的模型/程序壳，尚无自有美术。替换正式美术时**不得改动**：逻辑ID、数值（hp/伤害/速度）、行为键（orbit）、体型倍率与染色值 —— 依据 docs/v0.1/design/怪物设计.md §T1~§T3。逐房编成见同文档 §T5；明确没做到原作的六处见 §T6。</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="190" customHeight="1" s="38">
+      <c r="A54" s="90" t="inlineStr">
+        <is>
+          <t>ENM-MELEE-EXPEDITION03-INFECTED01</t>
+        </is>
+      </c>
+      <c r="B54" s="91" t="inlineStr">
+        <is>
+          <t>远征03_普通感染者</t>
+        </is>
+      </c>
+      <c r="C54" s="91" t="inlineStr">
+        <is>
+          <t>敌人</t>
+        </is>
+      </c>
+      <c r="D54" s="90" t="inlineStr">
+        <is>
+          <t>normal_melee</t>
+        </is>
+      </c>
+      <c r="E54" s="90" t="inlineStr">
+        <is>
+          <t>enm_melee_expedition03_infected01</t>
+        </is>
+      </c>
+      <c r="F54" s="90" t="inlineStr">
+        <is>
+          <t>root_3d</t>
+        </is>
+      </c>
+      <c r="G54" s="91" t="inlineStr">
+        <is>
+          <t>ENM-ECOSYSTEM-KIT-3D</t>
+        </is>
+      </c>
+      <c r="H54" s="91" t="inlineStr">
+        <is>
+          <t>top3d</t>
+        </is>
+      </c>
+      <c r="I54" s="90" t="inlineStr">
+        <is>
+          <t>T Pose / TPOSE_reference（单帧参考）</t>
+        </is>
+      </c>
+      <c r="J54" s="92" t="inlineStr">
+        <is>
+          <t>远征03（expedition_03）怪物美术；新模型，未投放</t>
+        </is>
+      </c>
+      <c r="K54" s="91" t="inlineStr">
+        <is>
+          <t>authored</t>
+        </is>
+      </c>
+      <c r="L54" s="90" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="M54" s="90" t="inlineStr">
+        <is>
+          <t>v002</t>
+        </is>
+      </c>
+      <c r="N54" s="91" t="inlineStr">
+        <is>
+          <t>创作高1.600m；臂展1.130m（原1.900m）；双臂从肩向外缩短50%；475面/475三角；389顶点；39网格；4材质；20骨；T Pose；512×512 NPC色盘/10×10/PaletteUV；运行展示尺寸未验</t>
+        </is>
+      </c>
+      <c r="O54" s="91" t="inlineStr">
+        <is>
+          <t>art_source/enemies/enemy_3d/enm_melee_expedition03_infected01/source/enm_melee_expedition03_infected01_model_v002.blend</t>
+        </is>
+      </c>
+      <c r="P54" s="90" t="inlineStr">
+        <is>
+          <t>用户2026-10-30要求手臂短一点；模型=art_source/enemies/enemy_3d/enm_melee_expedition03_infected01/source/enm_melee_expedition03_infected01_model_v002.blend；动作参考=art_source/enemies/enemy_3d/enm_melee_expedition03_infected01/source/enm_melee_expedition03_infected01_animation_v002.blend；SKEL-INFECTED01-002；契约=art_source/enemies/enemy_3d/enm_melee_expedition03_infected01/source/README.md；清单=art_source/enemies/enemy_3d/enm_melee_expedition03_infected01/source/enm_melee_expedition03_infected01_manifest_v002.json；双母版静止骨架签名7c4b4dc76f0787b8afdd1f6073da65cf6d9a04496cc26a4539a3d58ab3aa2e92；仅TPOSE_reference单帧；m/根缩放1/脚底Z=0；独立重开审计591/591通过exit0</t>
+        </is>
+      </c>
+      <c r="Q54" s="91" t="inlineStr">
+        <is>
+          <t>远征03,感染者,长舌,破衬衫,胖体,低多边形,Tpose</t>
+        </is>
+      </c>
+      <c r="R54" s="91">
+        <f>LOWER(TRIM(C54)&amp;"|"&amp;TRIM(D54)&amp;"|"&amp;TRIM(E54)&amp;"|"&amp;TRIM(F54)&amp;"|"&amp;TRIM(H54)&amp;"|"&amp;TRIM(I54))</f>
+        <v/>
+      </c>
+      <c r="S54" s="91">
+        <f>IF(COUNTIF($R$6:$R$54,R54)&gt;1,"重复","唯一")</f>
+        <v/>
+      </c>
+      <c r="T54" s="91" t="inlineStr">
+        <is>
+          <t>791b163e57fea9f088d7ff9ed7523d132cec9685da9661b8d1017c5c868dbe92</t>
+        </is>
+      </c>
+      <c r="U54" s="91" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="V54" s="93" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="W54" s="91" t="inlineStr">
+        <is>
+          <t>用户提供参考图，仅作本项目制作依据</t>
+        </is>
+      </c>
+      <c r="X54" s="94" t="inlineStr">
+        <is>
+          <t>远征03_普通感染者_中文资产管理</t>
+        </is>
+      </c>
+      <c r="Y54" s="92" t="inlineStr">
+        <is>
+          <t>2026-10-30 v002：按用户要求，双臂从肩x=±0.18m向外缩短50%，臂展1.900→1.130m；新骨架身份SKEL-INFECTED01-002。保持1.600m身高、475面/475三角、389顶点、39网格、4材质、20骨及T Pose。模型/动作双母版静止签名一致，保存后独立Blender重开审计591/591通过，0预期故障、0非预期错误；全部475面保持非零面积PaletteUV色格安全内区、活动与渲染UV一致、Closest插值、公共外链色板未打包。证据：I:\工作项目\shellstrom2\ShellStorm2-work\sessions\2026-10-30_expedition03_infected\v002\independent_audit.json及同目录front/side/back/overview_v002.png。共享NPC色板assets/art/shared/palette/npc_palette_10x10_512.png；分层源art_source/shared/palette/npc_palette_10x10_512_v001.psd。动作参考SHA-256=5b851072402a87c48dd05ee04cee02d5bd795ffea13f95dcb36c906b2480f125。旧v001制作源已移工程外备份；状态authored，仅制作源完成，未制作12态动作/GLB/运行Prefab，运行展示尺寸和Godot接入未验，不改既有33只egt怪物映射。</t>
         </is>
       </c>
     </row>
@@ -8187,17 +8315,17 @@
     <row r="427" ht="84.75" customHeight="1" s="38"/>
     <row r="429" ht="120" customHeight="1" s="38"/>
   </sheetData>
-  <autoFilter ref="A5:Y20"/>
+  <autoFilter ref="A5:Y54"/>
   <mergeCells count="2">
     <mergeCell ref="A1:X2"/>
     <mergeCell ref="A3:X3"/>
   </mergeCells>
-  <conditionalFormatting sqref="S6:S17">
+  <conditionalFormatting sqref="S6:S54">
     <cfRule type="containsText" rank="0" priority="2" equalAverage="0" operator="containsText" aboveAverage="0" dxfId="6" text="重复" percent="0" bottom="0">
       <formula>NOT(ISERROR(SEARCH("重复",S6)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K6:K17">
+  <conditionalFormatting sqref="K6:K54">
     <cfRule type="containsText" rank="0" priority="3" equalAverage="0" operator="containsText" aboveAverage="0" dxfId="7" text="已完成" percent="0" bottom="0">
       <formula>NOT(ISERROR(SEARCH("已完成",K6)))</formula>
     </cfRule>
@@ -8206,15 +8334,15 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation sqref="C6:C20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop">
+    <dataValidation sqref="C6:C54" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop">
       <formula1>"角色,敌人,武器,道具,场景,场景道具,基地资产包,UI,特效,音频"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation sqref="K6:K20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop">
+    <dataValidation sqref="K6:K54" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop">
       <formula1>"待制作,程序占位,已完成,原型已接入,弃用,旧资产已从正式基地移除,正式美术已接入,已优化并正式接入,Blender源已完成,已导入；优化完成,已从运行场景移除,白盒组件,design_only,authored,exported_pending_godot_validation,validated,active"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation sqref="L6:L20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop">
+    <dataValidation sqref="L6:L54" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop">
       <formula1>"P0,P1,P2,P3"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -8263,6 +8391,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="31.5" customHeight="1" s="38">
       <c r="A5" s="44" t="inlineStr">
         <is>
@@ -8850,6 +8979,7 @@
         </is>
       </c>
     </row>
+    <row r="18"/>
     <row r="19" ht="15" customHeight="1" s="38">
       <c r="A19" s="51" t="inlineStr">
         <is>
@@ -10615,12 +10745,12 @@
       </c>
       <c r="D59" s="37" t="inlineStr">
         <is>
-          <t>3.2s；保留身体曲线，手指不独立运动</t>
+          <t>3.2s；手部随前臂、脚部随小腿；无手指/手/脚骨</t>
         </is>
       </c>
       <c r="E59" s="37" t="inlineStr">
         <is>
-          <t>art_source/enemies/normal_enemy_3d/melee_chaser/source/animation/enm_melee_fungboar01_animation_v004.blend</t>
+          <t>art_source/enemies/normal_enemy_3d/melee_chaser/source/animation/enm_melee_fungboar01_animation_v005.blend</t>
         </is>
       </c>
       <c r="F59" s="37" t="inlineStr">
@@ -10635,12 +10765,12 @@
       </c>
       <c r="H59" s="37" t="inlineStr">
         <is>
-          <t>已重新蒙皮/导入/验收</t>
+          <t>v005源重开/重新导入/专项已验收</t>
         </is>
       </c>
       <c r="I59" s="37" t="inlineStr">
         <is>
-          <t>2026-10-09 v004减面与减骨：4552→1790三角，897顶点；36→20骨，移除16根手指骨，每手仅一根手骨；自然弯曲形状固定，手指权重合并至手骨并重新归一。512贴图/六段身体动作/12态/碰撞/受击闪色/2.4秒死亡保留。源重开、半帧蒙皮检查、运行专项及死亡视野真实渲染通过。</t>
+          <t>2026-10-30 v005减面减骨：1790→800三角、402原生顶点，20→16骨；删除左右Hand/Foot骨，手指骨原已移除；手部随前臂、脚部随小腿，腕踝固定，不再独立弯曲。模型v004/动作v005，骨架SKEL-MELEE-ZOMBIE01-004（签名4b0767495dde049f663598129f285158dd04bdbe309ef2a66e042b8d6db033bb）；六剪辑时长/循环与12态采样保留。名义展示1.3m/倍率0.70不变；静止绑定脚底Z=0，高1.893537m；待机首姿源高1.800935m（展示约1.26065m），不能把静止绑定高度与姿势高度混为一谈。双源重开、1266个四分之一帧蒙皮/地面检查通过（最低Z≥0.0004999m、单位姿势、Root静止、循环接缝0），GLB六段时长精确。近景细节因减面简化；未进行全程自穿插、滑步及目标设备性能验收。运行专项exit0（12态/6剪辑/16骨/800三角/碰撞不变）；801面负向对照exit1且仅预期预算错误；120Hz运行时1266采样地面最低+0.00003319m、Root静止；存活12姿态及死亡可见性真实渲染均exit0，无非预期脚本错误。证据：ShellStorm2-work/sessions/2026-10-30_melee_800/；GLB SHA-256=800f1be604c65de3c0b669d0082b4e434f70dcebf70aa0b46918d643844ef775（172668字节），共享原有贴图。</t>
         </is>
       </c>
     </row>
@@ -10662,12 +10792,12 @@
       </c>
       <c r="D60" s="37" t="inlineStr">
         <is>
-          <t>1.6s；保留身体曲线，手指不独立运动</t>
+          <t>1.6s；手部随前臂、脚部随小腿；无手指/手/脚骨</t>
         </is>
       </c>
       <c r="E60" s="37" t="inlineStr">
         <is>
-          <t>art_source/enemies/normal_enemy_3d/melee_chaser/source/animation/enm_melee_fungboar01_animation_v004.blend</t>
+          <t>art_source/enemies/normal_enemy_3d/melee_chaser/source/animation/enm_melee_fungboar01_animation_v005.blend</t>
         </is>
       </c>
       <c r="F60" s="37" t="inlineStr">
@@ -10682,12 +10812,12 @@
       </c>
       <c r="H60" s="37" t="inlineStr">
         <is>
-          <t>已重新蒙皮/导入/验收</t>
+          <t>v005源重开/重新导入/专项已验收</t>
         </is>
       </c>
       <c r="I60" s="37" t="inlineStr">
         <is>
-          <t>2026-10-09 v004减面与减骨：4552→1790三角，897顶点；36→20骨，移除16根手指骨，每手仅一根手骨；自然弯曲形状固定，手指权重合并至手骨并重新归一。512贴图/六段身体动作/12态/碰撞/受击闪色/2.4秒死亡保留。源重开、半帧蒙皮检查、运行专项及死亡视野真实渲染通过。</t>
+          <t>2026-10-30 v005减面减骨：1790→800三角、402原生顶点，20→16骨；删除左右Hand/Foot骨，手指骨原已移除；手部随前臂、脚部随小腿，腕踝固定，不再独立弯曲。模型v004/动作v005，骨架SKEL-MELEE-ZOMBIE01-004（签名4b0767495dde049f663598129f285158dd04bdbe309ef2a66e042b8d6db033bb）；六剪辑时长/循环与12态采样保留。名义展示1.3m/倍率0.70不变；静止绑定脚底Z=0，高1.893537m；待机首姿源高1.800935m（展示约1.26065m），不能把静止绑定高度与姿势高度混为一谈。双源重开、1266个四分之一帧蒙皮/地面检查通过（最低Z≥0.0004999m、单位姿势、Root静止、循环接缝0），GLB六段时长精确。近景细节因减面简化；未进行全程自穿插、滑步及目标设备性能验收。运行专项exit0（12态/6剪辑/16骨/800三角/碰撞不变）；801面负向对照exit1且仅预期预算错误；120Hz运行时1266采样地面最低+0.00003319m、Root静止；存活12姿态及死亡可见性真实渲染均exit0，无非预期脚本错误。证据：ShellStorm2-work/sessions/2026-10-30_melee_800/；GLB SHA-256=800f1be604c65de3c0b669d0082b4e434f70dcebf70aa0b46918d643844ef775（172668字节），共享原有贴图。</t>
         </is>
       </c>
     </row>
@@ -10709,12 +10839,12 @@
       </c>
       <c r="D61" s="37" t="inlineStr">
         <is>
-          <t>0.8s；保留身体曲线，手指不独立运动</t>
+          <t>0.8s；手部随前臂、脚部随小腿；无手指/手/脚骨</t>
         </is>
       </c>
       <c r="E61" s="37" t="inlineStr">
         <is>
-          <t>art_source/enemies/normal_enemy_3d/melee_chaser/source/animation/enm_melee_fungboar01_animation_v004.blend</t>
+          <t>art_source/enemies/normal_enemy_3d/melee_chaser/source/animation/enm_melee_fungboar01_animation_v005.blend</t>
         </is>
       </c>
       <c r="F61" s="37" t="inlineStr">
@@ -10729,12 +10859,12 @@
       </c>
       <c r="H61" s="37" t="inlineStr">
         <is>
-          <t>已重新蒙皮/导入/验收</t>
+          <t>v005源重开/重新导入/专项已验收</t>
         </is>
       </c>
       <c r="I61" s="37" t="inlineStr">
         <is>
-          <t>2026-10-09 v004减面与减骨：4552→1790三角，897顶点；36→20骨，移除16根手指骨，每手仅一根手骨；自然弯曲形状固定，手指权重合并至手骨并重新归一。512贴图/六段身体动作/12态/碰撞/受击闪色/2.4秒死亡保留。源重开、半帧蒙皮检查、运行专项及死亡视野真实渲染通过。</t>
+          <t>2026-10-30 v005减面减骨：1790→800三角、402原生顶点，20→16骨；删除左右Hand/Foot骨，手指骨原已移除；手部随前臂、脚部随小腿，腕踝固定，不再独立弯曲。模型v004/动作v005，骨架SKEL-MELEE-ZOMBIE01-004（签名4b0767495dde049f663598129f285158dd04bdbe309ef2a66e042b8d6db033bb）；六剪辑时长/循环与12态采样保留。名义展示1.3m/倍率0.70不变；静止绑定脚底Z=0，高1.893537m；待机首姿源高1.800935m（展示约1.26065m），不能把静止绑定高度与姿势高度混为一谈。双源重开、1266个四分之一帧蒙皮/地面检查通过（最低Z≥0.0004999m、单位姿势、Root静止、循环接缝0），GLB六段时长精确。近景细节因减面简化；未进行全程自穿插、滑步及目标设备性能验收。运行专项exit0（12态/6剪辑/16骨/800三角/碰撞不变）；801面负向对照exit1且仅预期预算错误；120Hz运行时1266采样地面最低+0.00003319m、Root静止；存活12姿态及死亡可见性真实渲染均exit0，无非预期脚本错误。证据：ShellStorm2-work/sessions/2026-10-30_melee_800/；GLB SHA-256=800f1be604c65de3c0b669d0082b4e434f70dcebf70aa0b46918d643844ef775（172668字节），共享原有贴图。</t>
         </is>
       </c>
     </row>
@@ -10756,12 +10886,12 @@
       </c>
       <c r="D62" s="37" t="inlineStr">
         <is>
-          <t>1.7s；保留身体曲线，手指不独立运动</t>
+          <t>1.7s；手部随前臂、脚部随小腿；无手指/手/脚骨</t>
         </is>
       </c>
       <c r="E62" s="37" t="inlineStr">
         <is>
-          <t>art_source/enemies/normal_enemy_3d/melee_chaser/source/animation/enm_melee_fungboar01_animation_v004.blend</t>
+          <t>art_source/enemies/normal_enemy_3d/melee_chaser/source/animation/enm_melee_fungboar01_animation_v005.blend</t>
         </is>
       </c>
       <c r="F62" s="37" t="inlineStr">
@@ -10776,12 +10906,12 @@
       </c>
       <c r="H62" s="37" t="inlineStr">
         <is>
-          <t>已重新蒙皮/导入/验收</t>
+          <t>v005源重开/重新导入/专项已验收</t>
         </is>
       </c>
       <c r="I62" s="37" t="inlineStr">
         <is>
-          <t>2026-10-09 v004减面与减骨：4552→1790三角，897顶点；36→20骨，移除16根手指骨，每手仅一根手骨；自然弯曲形状固定，手指权重合并至手骨并重新归一。512贴图/六段身体动作/12态/碰撞/受击闪色/2.4秒死亡保留。源重开、半帧蒙皮检查、运行专项及死亡视野真实渲染通过。</t>
+          <t>2026-10-30 v005减面减骨：1790→800三角、402原生顶点，20→16骨；删除左右Hand/Foot骨，手指骨原已移除；手部随前臂、脚部随小腿，腕踝固定，不再独立弯曲。模型v004/动作v005，骨架SKEL-MELEE-ZOMBIE01-004（签名4b0767495dde049f663598129f285158dd04bdbe309ef2a66e042b8d6db033bb）；六剪辑时长/循环与12态采样保留。名义展示1.3m/倍率0.70不变；静止绑定脚底Z=0，高1.893537m；待机首姿源高1.800935m（展示约1.26065m），不能把静止绑定高度与姿势高度混为一谈。双源重开、1266个四分之一帧蒙皮/地面检查通过（最低Z≥0.0004999m、单位姿势、Root静止、循环接缝0），GLB六段时长精确。近景细节因减面简化；未进行全程自穿插、滑步及目标设备性能验收。运行专项exit0（12态/6剪辑/16骨/800三角/碰撞不变）；801面负向对照exit1且仅预期预算错误；120Hz运行时1266采样地面最低+0.00003319m、Root静止；存活12姿态及死亡可见性真实渲染均exit0，无非预期脚本错误。证据：ShellStorm2-work/sessions/2026-10-30_melee_800/；GLB SHA-256=800f1be604c65de3c0b669d0082b4e434f70dcebf70aa0b46918d643844ef775（172668字节），共享原有贴图。</t>
         </is>
       </c>
     </row>
@@ -10803,12 +10933,12 @@
       </c>
       <c r="D63" s="37" t="inlineStr">
         <is>
-          <t>0.8s；保留身体曲线，手指不独立运动</t>
+          <t>0.8s；手部随前臂、脚部随小腿；无手指/手/脚骨</t>
         </is>
       </c>
       <c r="E63" s="37" t="inlineStr">
         <is>
-          <t>art_source/enemies/normal_enemy_3d/melee_chaser/source/animation/enm_melee_fungboar01_animation_v004.blend</t>
+          <t>art_source/enemies/normal_enemy_3d/melee_chaser/source/animation/enm_melee_fungboar01_animation_v005.blend</t>
         </is>
       </c>
       <c r="F63" s="37" t="inlineStr">
@@ -10823,12 +10953,12 @@
       </c>
       <c r="H63" s="37" t="inlineStr">
         <is>
-          <t>已重新蒙皮/导入/验收</t>
+          <t>v005源重开/重新导入/专项已验收</t>
         </is>
       </c>
       <c r="I63" s="37" t="inlineStr">
         <is>
-          <t>2026-10-09 v004减面与减骨：4552→1790三角，897顶点；36→20骨，移除16根手指骨，每手仅一根手骨；自然弯曲形状固定，手指权重合并至手骨并重新归一。512贴图/六段身体动作/12态/碰撞/受击闪色/2.4秒死亡保留。源重开、半帧蒙皮检查、运行专项及死亡视野真实渲染通过。</t>
+          <t>2026-10-30 v005减面减骨：1790→800三角、402原生顶点，20→16骨；删除左右Hand/Foot骨，手指骨原已移除；手部随前臂、脚部随小腿，腕踝固定，不再独立弯曲。模型v004/动作v005，骨架SKEL-MELEE-ZOMBIE01-004（签名4b0767495dde049f663598129f285158dd04bdbe309ef2a66e042b8d6db033bb）；六剪辑时长/循环与12态采样保留。名义展示1.3m/倍率0.70不变；静止绑定脚底Z=0，高1.893537m；待机首姿源高1.800935m（展示约1.26065m），不能把静止绑定高度与姿势高度混为一谈。双源重开、1266个四分之一帧蒙皮/地面检查通过（最低Z≥0.0004999m、单位姿势、Root静止、循环接缝0），GLB六段时长精确。近景细节因减面简化；未进行全程自穿插、滑步及目标设备性能验收。运行专项exit0（12态/6剪辑/16骨/800三角/碰撞不变）；801面负向对照exit1且仅预期预算错误；120Hz运行时1266采样地面最低+0.00003319m、Root静止；存活12姿态及死亡可见性真实渲染均exit0，无非预期脚本错误。证据：ShellStorm2-work/sessions/2026-10-30_melee_800/；GLB SHA-256=800f1be604c65de3c0b669d0082b4e434f70dcebf70aa0b46918d643844ef775（172668字节），共享原有贴图。</t>
         </is>
       </c>
     </row>
@@ -10850,12 +10980,12 @@
       </c>
       <c r="D64" s="37" t="inlineStr">
         <is>
-          <t>2.4s；保留身体曲线，手指不独立运动</t>
+          <t>2.4s；手部随前臂、脚部随小腿；无手指/手/脚骨</t>
         </is>
       </c>
       <c r="E64" s="37" t="inlineStr">
         <is>
-          <t>art_source/enemies/normal_enemy_3d/melee_chaser/source/animation/enm_melee_fungboar01_animation_v004.blend</t>
+          <t>art_source/enemies/normal_enemy_3d/melee_chaser/source/animation/enm_melee_fungboar01_animation_v005.blend</t>
         </is>
       </c>
       <c r="F64" s="37" t="inlineStr">
@@ -10870,12 +11000,12 @@
       </c>
       <c r="H64" s="37" t="inlineStr">
         <is>
-          <t>已重新蒙皮/导入/验收</t>
+          <t>v005源重开/重新导入/专项已验收</t>
         </is>
       </c>
       <c r="I64" s="37" t="inlineStr">
         <is>
-          <t>2026-10-09 v004减面与减骨：4552→1790三角，897顶点；36→20骨，移除16根手指骨，每手仅一根手骨；自然弯曲形状固定，手指权重合并至手骨并重新归一。512贴图/六段身体动作/12态/碰撞/受击闪色/2.4秒死亡保留。源重开、半帧蒙皮检查、运行专项及死亡视野真实渲染通过。</t>
+          <t>2026-10-30 v005减面减骨：1790→800三角、402原生顶点，20→16骨；删除左右Hand/Foot骨，手指骨原已移除；手部随前臂、脚部随小腿，腕踝固定，不再独立弯曲。模型v004/动作v005，骨架SKEL-MELEE-ZOMBIE01-004（签名4b0767495dde049f663598129f285158dd04bdbe309ef2a66e042b8d6db033bb）；六剪辑时长/循环与12态采样保留。名义展示1.3m/倍率0.70不变；静止绑定脚底Z=0，高1.893537m；待机首姿源高1.800935m（展示约1.26065m），不能把静止绑定高度与姿势高度混为一谈。双源重开、1266个四分之一帧蒙皮/地面检查通过（最低Z≥0.0004999m、单位姿势、Root静止、循环接缝0），GLB六段时长精确。近景细节因减面简化；未进行全程自穿插、滑步及目标设备性能验收。运行专项exit0（12态/6剪辑/16骨/800三角/碰撞不变）；801面负向对照exit1且仅预期预算错误；120Hz运行时1266采样地面最低+0.00003319m、Root静止；存活12姿态及死亡可见性真实渲染均exit0，无非预期脚本错误。证据：ShellStorm2-work/sessions/2026-10-30_melee_800/；GLB SHA-256=800f1be604c65de3c0b669d0082b4e434f70dcebf70aa0b46918d643844ef775（172668字节），共享原有贴图。</t>
         </is>
       </c>
     </row>
@@ -10931,6 +11061,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="30" customHeight="1" s="38">
       <c r="A4" s="69" t="inlineStr">
         <is>
@@ -11192,12 +11323,12 @@
       </c>
       <c r="E7" s="65" t="inlineStr">
         <is>
-          <t>art_source/enemies/normal_enemy_3d/melee_chaser/source/model/enm_melee_fungboar01_model_v003.blend; art_source/enemies/normal_enemy_3d/melee_chaser/source/animation/enm_melee_fungboar01_animation_v004.blend</t>
+          <t>art_source/enemies/normal_enemy_3d/melee_chaser/source/model/enm_melee_fungboar01_model_v004.blend; art_source/enemies/normal_enemy_3d/melee_chaser/source/animation/enm_melee_fungboar01_animation_v005.blend</t>
         </is>
       </c>
       <c r="F7" s="41" t="inlineStr">
         <is>
-          <t>六段Blender剪辑按12态采样；20骨，每手一骨</t>
+          <t>六段Blender剪辑按12态采样；16骨；无手指/手/脚骨，腿部仅大腿/小腿</t>
         </is>
       </c>
       <c r="G7" s="65" t="inlineStr">
@@ -11222,7 +11353,7 @@
       </c>
       <c r="K7" s="65" t="inlineStr">
         <is>
-          <t>源高1.857143m/游戏1.3m；1790三角/897顶点；20骨；512贴图</t>
+          <t>名义展示1.3m/倍率0.70；静止绑定高1.893537m；800三角/402顶点；16骨；512贴图；6剪辑</t>
         </is>
       </c>
       <c r="L7" s="41" t="inlineStr">
@@ -11242,12 +11373,13 @@
       </c>
       <c r="O7" s="65" t="inlineStr">
         <is>
-          <t>v004</t>
+          <t>v005</t>
         </is>
       </c>
       <c r="P7" s="41" t="inlineStr">
         <is>
-          <t>无碰撞；Enemy3D 持有碰撞/AI/伤害/掉落。碰撞体尺寸沿用旧程序网格口径（1.02/1.30），与模型几何（0.641/1.857）不一致，待拍板后再收紧。显示名 小菌猪 → 小僵尸。；2026-10-09 v004减面与减骨：4552→1790三角，897顶点；36→20骨，移除16根手指骨，每手仅一根手骨；自然弯曲形状固定，手指权重合并至手骨并重新归一。512贴图/六段身体动作/12态/碰撞/受击闪色/2.4秒死亡保留。源重开、半帧蒙皮检查、运行专项及死亡视野真实渲染通过。</t>
+          <t>无碰撞；Enemy3D 持有碰撞/AI/伤害/掉落。碰撞体尺寸沿用旧程序网格口径（1.02/1.30），与模型几何（0.641/1.857）不一致，待拍板后再收紧。显示名 小菌猪 → 小僵尸。；2026-10-09 v004减面与减骨：4552→1790三角，897顶点；36→20骨，移除16根手指骨，每手仅一根手骨；自然弯曲形状固定，手指权重合并至手骨并重新归一。512贴图/六段身体动作/12态/碰撞/受击闪色/2.4秒死亡保留。源重开、半帧蒙皮检查、运行专项及死亡视野真实渲染通过。
+2026-10-30 v005减面减骨：1790→800三角、402原生顶点，20→16骨；删除左右Hand/Foot骨，手指骨原已移除；手部随前臂、脚部随小腿，腕踝固定，不再独立弯曲。模型v004/动作v005，骨架SKEL-MELEE-ZOMBIE01-004（签名4b0767495dde049f663598129f285158dd04bdbe309ef2a66e042b8d6db033bb）；六剪辑时长/循环与12态采样保留。名义展示1.3m/倍率0.70不变；静止绑定脚底Z=0，高1.893537m；待机首姿源高1.800935m（展示约1.26065m），不能把静止绑定高度与姿势高度混为一谈。双源重开、1266个四分之一帧蒙皮/地面检查通过（最低Z≥0.0004999m、单位姿势、Root静止、循环接缝0），GLB六段时长精确。近景细节因减面简化；未进行全程自穿插、滑步及目标设备性能验收。运行专项exit0（12态/6剪辑/16骨/800三角/碰撞不变）；801面负向对照exit1且仅预期预算错误；120Hz运行时1266采样地面最低+0.00003319m、Root静止；存活12姿态及死亡可见性真实渲染均exit0，无非预期脚本错误。证据：ShellStorm2-work/sessions/2026-10-30_melee_800/；GLB SHA-256=800f1be604c65de3c0b669d0082b4e434f70dcebf70aa0b46918d643844ef775（172668字节），共享原有贴图。</t>
         </is>
       </c>
     </row>
@@ -11528,7 +11660,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:G65"/>
+  <dimension ref="A1:G69"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="10.359375" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="16.71" customWidth="1" style="37" min="1" max="1"/>
@@ -13520,6 +13652,154 @@
         </is>
       </c>
     </row>
+    <row r="66" s="38">
+      <c r="A66" s="95" t="inlineStr">
+        <is>
+          <t>v0.1.24</t>
+        </is>
+      </c>
+      <c r="B66" s="95" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="C66" s="96" t="inlineStr">
+        <is>
+          <t>新怪物设计登记</t>
+        </is>
+      </c>
+      <c r="D66" s="96" t="inlineStr">
+        <is>
+          <t>远征03 普通感染者</t>
+        </is>
+      </c>
+      <c r="E66" s="96" t="inlineStr">
+        <is>
+          <t>ENM-MELEE-EXPEDITION03-INFECTED01新增r54；约1.6m、T Pose、≤500面、最多四材质，新增NPC色盘并按场景PaletteUV规则制作。状态design_only；源路径art_source/enemies/enemy_3d/enm_melee_expedition03_infected01/source/enm_melee_expedition03_infected01_model_v001.blend。</t>
+        </is>
+      </c>
+      <c r="F66" s="96" t="inlineStr">
+        <is>
+          <t>仅Blender制作源；未接入Godot或替换现有怪物映射</t>
+        </is>
+      </c>
+      <c r="G66" s="96" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" s="38">
+      <c r="A67" s="95" t="inlineStr">
+        <is>
+          <t>v0.1.25</t>
+        </is>
+      </c>
+      <c r="B67" s="95" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="C67" s="96" t="inlineStr">
+        <is>
+          <t>怪物T Pose母版完成</t>
+        </is>
+      </c>
+      <c r="D67" s="96" t="inlineStr">
+        <is>
+          <t>远征03 普通感染者</t>
+        </is>
+      </c>
+      <c r="E67" s="96" t="inlineStr">
+        <is>
+          <t>ENM-MELEE-EXPEDITION03-INFECTED01 design_only→authored；创作高1.600m；475面/475三角；389顶点；39网格；4材质；20骨；T Pose；512×512 NPC色盘/10×10/PaletteUV；运行展示尺寸未验；双母版、共享NPC色板及PaletteUV原生重开验收；本资产source/README.md；enm_melee_expedition03_infected01_manifest_v001.json；双母版静止骨架签名e2a7e46d9631865f1b9add928d36016929d06a3935f27a5fda990c454b3b2267；只含TPOSE_reference单帧参考；单位m、根缩放1、脚底Z=0；当前原生独立审计588/588通过exit0</t>
+        </is>
+      </c>
+      <c r="F67" s="96" t="inlineStr">
+        <is>
+          <t>仅Blender制作源；未接入Godot或替换现有怪物映射</t>
+        </is>
+      </c>
+      <c r="G67" s="96" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" s="38">
+      <c r="A68" s="95" t="inlineStr">
+        <is>
+          <t>v0.1.26</t>
+        </is>
+      </c>
+      <c r="B68" s="95" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="C68" s="96" t="inlineStr">
+        <is>
+          <t>感染者手臂缩短v002</t>
+        </is>
+      </c>
+      <c r="D68" s="96" t="inlineStr">
+        <is>
+          <t>远征03 普通感染者</t>
+        </is>
+      </c>
+      <c r="E68" s="96" t="inlineStr">
+        <is>
+          <t>ENM-MELEE-EXPEDITION03-INFECTED01；双臂从肩向外缩短50%，臂展1.900→1.130m，仍为1.600m/475三角/389顶点/4材质/20骨/T Pose；骨架SKEL-INFECTED01-002；双母版签名7c4b4dc76f0787b8afdd1f6073da65cf6d9a04496cc26a4539a3d58ab3aa2e92；原生重开591/591通过；仅更新r54版本、双源路径、签名和SHA，状态authored。</t>
+        </is>
+      </c>
+      <c r="F68" s="96" t="inlineStr">
+        <is>
+          <t>仅Blender制作源；未接入Godot或替换现有怪物映射</t>
+        </is>
+      </c>
+      <c r="G68" s="96" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" s="38">
+      <c r="A69" s="95" t="inlineStr">
+        <is>
+          <t>v0.1.27</t>
+        </is>
+      </c>
+      <c r="B69" s="95" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="C69" s="96" t="inlineStr">
+        <is>
+          <t>小僵尸减面减骨v005</t>
+        </is>
+      </c>
+      <c r="D69" s="96" t="inlineStr">
+        <is>
+          <t>小僵尸</t>
+        </is>
+      </c>
+      <c r="E69" s="96" t="inlineStr">
+        <is>
+          <t>2026-10-30 v005减面减骨：1790→800三角、402原生顶点，20→16骨；删除左右Hand/Foot骨，手指骨原已移除；手部随前臂、脚部随小腿，腕踝固定，不再独立弯曲。模型v004/动作v005，骨架SKEL-MELEE-ZOMBIE01-004（签名4b0767495dde049f663598129f285158dd04bdbe309ef2a66e042b8d6db033bb）；六剪辑时长/循环与12态采样保留。名义展示1.3m/倍率0.70不变；静止绑定脚底Z=0，高1.893537m；待机首姿源高1.800935m（展示约1.26065m），不能把静止绑定高度与姿势高度混为一谈。双源重开、1266个四分之一帧蒙皮/地面检查通过（最低Z≥0.0004999m、单位姿势、Root静止、循环接缝0），GLB六段时长精确。近景细节因减面简化；未进行全程自穿插、滑步及目标设备性能验收。运行专项exit0（12态/6剪辑/16骨/800三角/碰撞不变）；801面负向对照exit1且仅预期预算错误；120Hz运行时1266采样地面最低+0.00003319m、Root静止；存活12姿态及死亡可见性真实渲染均exit0，无非预期脚本错误。证据：ShellStorm2-work/sessions/2026-10-30_melee_800/；GLB SHA-256=800f1be604c65de3c0b669d0082b4e434f70dcebf70aa0b46918d643844ef775（172668字节），共享原有贴图。</t>
+        </is>
+      </c>
+      <c r="F69" s="96" t="inlineStr">
+        <is>
+          <t>仅表现资产；AssetID、逻辑ID、尺寸、碰撞、AI、伤害和掉落规则不变。</t>
+        </is>
+      </c>
+      <c r="G69" s="96" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A3:G3"/>

</xml_diff>